<commit_message>
test add vlan 60
</commit_message>
<xml_diff>
--- a/network-config.xlsx
+++ b/network-config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user002\netdevops-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0DD3A71-F5E1-456B-B34B-FD49631D9C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C9A7D96-0A7F-47B6-965B-0EB28A09E4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="166">
   <si>
     <t>NetDevOps Network Configuration</t>
   </si>
@@ -522,6 +522,15 @@
   </si>
   <si>
     <t>10.10.99.12</t>
+  </si>
+  <si>
+    <t>ENGINEER</t>
+  </si>
+  <si>
+    <t>10.10.60.0/24</t>
+  </si>
+  <si>
+    <t>10.10.60.1</t>
   </si>
 </sst>
 </file>
@@ -3081,10 +3090,18 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="B8" s="5">
+        <v>60</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>165</v>
+      </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>

</xml_diff>

<commit_message>
add vlan 50 60
</commit_message>
<xml_diff>
--- a/network-config.xlsx
+++ b/network-config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user002\netdevops-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBE4F76-52A1-4801-96E1-9C5AA5814902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DF2705-BBC6-4999-9303-0FFADB32616D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -397,13 +397,13 @@
     <t>ENGINEER</t>
   </si>
   <si>
-    <t>10.10.60.90/24</t>
-  </si>
-  <si>
     <t>10.10.60.1</t>
   </si>
   <si>
     <t>PC-ENGINEER</t>
+  </si>
+  <si>
+    <t>10.10.60.0/24</t>
   </si>
 </sst>
 </file>
@@ -1130,10 +1130,10 @@
         <v>120</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>30</v>
@@ -1142,7 +1142,7 @@
         <v>48</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H8" s="3" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
test remove vlan 60
</commit_message>
<xml_diff>
--- a/network-config.xlsx
+++ b/network-config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user002\netdevops-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DF2705-BBC6-4999-9303-0FFADB32616D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C08CBE5F-4C23-4B40-A17E-EAD1020325B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="120">
   <si>
     <t>VLAN ID</t>
   </si>
@@ -392,18 +392,6 @@
   </si>
   <si>
     <t>PC-FINANCE</t>
-  </si>
-  <si>
-    <t>ENGINEER</t>
-  </si>
-  <si>
-    <t>10.10.60.1</t>
-  </si>
-  <si>
-    <t>PC-ENGINEER</t>
-  </si>
-  <si>
-    <t>10.10.60.0/24</t>
   </si>
 </sst>
 </file>
@@ -1123,30 +1111,14 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="21.95" customHeight="1">
-      <c r="A8" s="3">
-        <v>60</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="H8" s="3" t="b">
-        <v>1</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
       <c r="J8" s="6" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
rm vlan 60 v2
</commit_message>
<xml_diff>
--- a/network-config.xlsx
+++ b/network-config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user002\netdevops-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4592ED8C-C925-47B9-B55C-F293B1901ADC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7CE667-C683-49F2-9098-8D824A579F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="120">
   <si>
     <t>VLAN ID</t>
   </si>
@@ -392,18 +392,6 @@
   </si>
   <si>
     <t>PC-FINANCE</t>
-  </si>
-  <si>
-    <t>ENGINEER</t>
-  </si>
-  <si>
-    <t>10.10.60.1</t>
-  </si>
-  <si>
-    <t>PC-ENGINEER</t>
-  </si>
-  <si>
-    <t>10.10.60.0/24</t>
   </si>
 </sst>
 </file>
@@ -1123,30 +1111,14 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="21.95" customHeight="1">
-      <c r="A8" s="3">
-        <v>60</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="H8" s="3" t="b">
-        <v>1</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
       <c r="J8" s="6" t="s">
         <v>5</v>
       </c>

</xml_diff>

<commit_message>
adad vlan 60 v2
</commit_message>
<xml_diff>
--- a/network-config.xlsx
+++ b/network-config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user002\netdevops-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7CE667-C683-49F2-9098-8D824A579F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2800B79-76EF-4FE6-95B0-0CE3475AFCEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="124">
   <si>
     <t>VLAN ID</t>
   </si>
@@ -392,6 +392,18 @@
   </si>
   <si>
     <t>PC-FINANCE</t>
+  </si>
+  <si>
+    <t>ENGINEER</t>
+  </si>
+  <si>
+    <t>10.10.60.1</t>
+  </si>
+  <si>
+    <t>PC-ENGINEER</t>
+  </si>
+  <si>
+    <t>10.10.60.0/24</t>
   </si>
 </sst>
 </file>
@@ -1111,14 +1123,30 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="21.95" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="A8" s="3">
+        <v>60</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="H8" s="3" t="b">
+        <v>1</v>
+      </c>
       <c r="J8" s="6" t="s">
         <v>5</v>
       </c>

</xml_diff>